<commit_message>
Created vulnerability mapping for CWE 1233 examples
</commit_message>
<xml_diff>
--- a/CWE_Examples/CWE-1233/CWE-1233-vulnerability-mapping.xlsx
+++ b/CWE_Examples/CWE-1233/CWE-1233-vulnerability-mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parks\OneDrive\Documents\UC\Summer Research\DetectRTL\CWE_Examples\CWE-1233\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parks\OneDrive\Documents\UC\Research\DetectRTL\CWE_Examples\CWE-1233\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{278CF804-1647-47A1-9CF7-3D006C44F229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89EF08C7-652A-4032-986F-29856C98A7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
updated vulnerability mapping for cwe 1233 examples
</commit_message>
<xml_diff>
--- a/CWE_Examples/CWE-1233/CWE-1233-vulnerability-mapping.xlsx
+++ b/CWE_Examples/CWE-1233/CWE-1233-vulnerability-mapping.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parks\OneDrive\Documents\UC\Research\DetectRTL\CWE_Examples\CWE-1233\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89EF08C7-652A-4032-986F-29856C98A7A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E569258-5A1E-4411-8896-FBBEECC8555F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Detailed Results" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="98">
   <si>
     <t>File Name</t>
   </si>
@@ -193,13 +194,139 @@
   </si>
   <si>
     <t>Secure: All security sensitive register assignments are protected</t>
+  </si>
+  <si>
+    <t>rdata is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>Assignment Missing Lock Bit Protection</t>
+  </si>
+  <si>
+    <t>CWE-1233</t>
+  </si>
+  <si>
+    <t>CWE_1233_example_9_vulnerable_parsed.json</t>
+  </si>
+  <si>
+    <t>data is assigned without correct lock bit enforcement</t>
+  </si>
+  <si>
+    <t>Incorrect Lock Enforcement</t>
+  </si>
+  <si>
+    <t>CWE_1233_example_8_vulnerable_parsed.json</t>
+  </si>
+  <si>
+    <t>newMessage is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>startHash is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>CWE_1233_example_6_vulnerable_parsed.json</t>
+  </si>
+  <si>
+    <t>CWE_1233_example_5_vulnerable_parsed.json</t>
+  </si>
+  <si>
+    <t>acct_mem is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>CWE_1233_example_4_vulnerable_parsed.json</t>
+  </si>
+  <si>
+    <t>key_reg2 is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>CWE_1233_example_3_vulnerable_parsed.json</t>
+  </si>
+  <si>
+    <t>key_reg1 is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>key_reg0 is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>CWE_1233_example_2_vulnerable_parsed.json</t>
+  </si>
+  <si>
+    <t>CWE_1233_example_1_vulnerable_parsed.json</t>
+  </si>
+  <si>
+    <t>end_reg is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>key_sel is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>CWE_1233_example_10_vulnerable_parsed.json</t>
+  </si>
+  <si>
+    <t>start is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>state is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>p_c is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Line Number</t>
+  </si>
+  <si>
+    <t>Vulnerability Type</t>
+  </si>
+  <si>
+    <t>Related CWE</t>
+  </si>
+  <si>
+    <t>start_reg is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>length_reg is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>source_addr_lsb_reg is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>dest_addr_lsb_reg is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>dest_addr_mdb_reg is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>done_reg is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>core_lock_reg is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>source_addr_msb_reg is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>block_reg is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>fuse_req_o is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>fuse_addr_o is assigned without lock bit protection</t>
+  </si>
+  <si>
+    <t>CWE_1233_example_7_vulnerable_parsed.json</t>
+  </si>
+  <si>
+    <t>msg_in is assigned without lock bit protection</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -215,16 +342,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -232,11 +376,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -256,6 +415,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1764,4 +1928,2020 @@
     <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A906EDC6-4E6A-459E-A629-5A5E7FE38FCA}">
+  <dimension ref="A1:E126"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="41.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="51.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" s="9">
+        <v>108</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" s="9">
+        <v>120</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="9">
+        <v>102</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="9">
+        <v>144</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="9">
+        <v>132</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="9">
+        <v>134</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="9">
+        <v>136</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" s="9">
+        <v>138</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="9">
+        <v>140</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="9">
+        <v>142</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" s="9">
+        <v>144</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="9">
+        <v>146</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="9">
+        <v>148</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="9">
+        <v>163</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D17" s="9">
+        <v>165</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D18" s="9">
+        <v>167</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D19" s="9">
+        <v>169</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="9">
+        <v>171</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D21" s="9">
+        <v>173</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22" s="9">
+        <v>175</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D23" s="9">
+        <v>177</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="9">
+        <v>179</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" s="9">
+        <v>181</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="D27" s="9">
+        <v>133</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="29" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D29" s="9">
+        <v>259</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D30" s="9">
+        <v>262</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" s="9">
+        <v>264</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D32" s="9">
+        <v>266</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="34" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D34" s="9">
+        <v>83</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D35" s="9">
+        <v>85</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D36" s="9">
+        <v>99</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D37" s="9">
+        <v>101</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B39" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D39" s="9">
+        <v>108</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D40" s="9">
+        <v>139</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D42" s="9">
+        <v>156</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D43" s="9">
+        <v>158</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B44" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D44" s="9">
+        <v>160</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B45" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D45" s="9">
+        <v>162</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B47" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D47" s="9">
+        <v>218</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B48" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D48" s="9">
+        <v>220</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B49" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D49" s="9">
+        <v>222</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B50" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D50" s="9">
+        <v>224</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D51" s="9">
+        <v>226</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D52" s="9">
+        <v>228</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D53" s="9">
+        <v>230</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D54" s="9">
+        <v>232</v>
+      </c>
+      <c r="E54" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D55" s="9">
+        <v>234</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D56" s="9">
+        <v>236</v>
+      </c>
+      <c r="E56" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D57" s="9">
+        <v>238</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B58" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D58" s="9">
+        <v>240</v>
+      </c>
+      <c r="E58" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D59" s="9">
+        <v>242</v>
+      </c>
+      <c r="E59" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B60" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D60" s="9">
+        <v>244</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D61" s="9">
+        <v>246</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B62" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C62" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D62" s="9">
+        <v>248</v>
+      </c>
+      <c r="E62" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C63" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D63" s="9">
+        <v>250</v>
+      </c>
+      <c r="E63" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B64" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C64" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D64" s="9">
+        <v>252</v>
+      </c>
+      <c r="E64" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C65" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D65" s="9">
+        <v>254</v>
+      </c>
+      <c r="E65" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B66" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C66" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D66" s="9">
+        <v>256</v>
+      </c>
+      <c r="E66" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B67" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D67" s="9">
+        <v>258</v>
+      </c>
+      <c r="E67" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B68" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C68" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D68" s="9">
+        <v>260</v>
+      </c>
+      <c r="E68" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B69" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C69" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D69" s="9">
+        <v>262</v>
+      </c>
+      <c r="E69" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B70" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C70" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D70" s="9">
+        <v>264</v>
+      </c>
+      <c r="E70" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B71" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C71" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D71" s="9">
+        <v>266</v>
+      </c>
+      <c r="E71" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B72" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D72" s="9">
+        <v>268</v>
+      </c>
+      <c r="E72" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B73" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C73" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D73" s="9">
+        <v>270</v>
+      </c>
+      <c r="E73" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B74" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C74" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D74" s="9">
+        <v>272</v>
+      </c>
+      <c r="E74" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B75" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C75" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D75" s="9">
+        <v>274</v>
+      </c>
+      <c r="E75" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B76" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C76" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D76" s="9">
+        <v>276</v>
+      </c>
+      <c r="E76" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B77" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C77" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D77" s="9">
+        <v>278</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B78" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C78" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D78" s="9">
+        <v>280</v>
+      </c>
+      <c r="E78" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B79" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C79" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D79" s="9">
+        <v>282</v>
+      </c>
+      <c r="E79" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B80" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C80" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D80" s="9">
+        <v>284</v>
+      </c>
+      <c r="E80" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B81" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C81" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D81" s="9">
+        <v>286</v>
+      </c>
+      <c r="E81" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B82" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C82" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D82" s="9">
+        <v>288</v>
+      </c>
+      <c r="E82" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B83" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C83" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D83" s="9">
+        <v>290</v>
+      </c>
+      <c r="E83" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B84" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C84" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D84" s="9">
+        <v>292</v>
+      </c>
+      <c r="E84" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B85" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C85" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D85" s="9">
+        <v>294</v>
+      </c>
+      <c r="E85" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B86" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C86" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D86" s="9">
+        <v>296</v>
+      </c>
+      <c r="E86" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B87" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C87" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D87" s="9">
+        <v>298</v>
+      </c>
+      <c r="E87" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B88" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C88" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D88" s="9">
+        <v>300</v>
+      </c>
+      <c r="E88" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B89" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C89" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D89" s="9">
+        <v>302</v>
+      </c>
+      <c r="E89" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B90" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C90" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D90" s="9">
+        <v>304</v>
+      </c>
+      <c r="E90" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B91" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C91" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D91" s="9">
+        <v>306</v>
+      </c>
+      <c r="E91" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B92" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C92" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D92" s="9">
+        <v>308</v>
+      </c>
+      <c r="E92" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B93" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C93" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D93" s="9">
+        <v>310</v>
+      </c>
+      <c r="E93" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C94" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D94" s="9">
+        <v>312</v>
+      </c>
+      <c r="E94" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B95" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C95" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D95" s="9">
+        <v>314</v>
+      </c>
+      <c r="E95" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B96" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C96" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D96" s="9">
+        <v>316</v>
+      </c>
+      <c r="E96" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B97" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C97" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D97" s="9">
+        <v>318</v>
+      </c>
+      <c r="E97" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B98" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C98" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D98" s="9">
+        <v>320</v>
+      </c>
+      <c r="E98" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B99" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C99" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D99" s="9">
+        <v>322</v>
+      </c>
+      <c r="E99" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B100" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C100" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D100" s="9">
+        <v>324</v>
+      </c>
+      <c r="E100" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B101" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C101" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D101" s="9">
+        <v>326</v>
+      </c>
+      <c r="E101" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B102" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C102" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D102" s="9">
+        <v>328</v>
+      </c>
+      <c r="E102" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B103" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C103" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D103" s="9">
+        <v>330</v>
+      </c>
+      <c r="E103" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B104" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C104" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D104" s="9">
+        <v>332</v>
+      </c>
+      <c r="E104" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B105" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C105" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D105" s="9">
+        <v>334</v>
+      </c>
+      <c r="E105" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A106" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B106" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C106" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D106" s="9">
+        <v>336</v>
+      </c>
+      <c r="E106" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A107" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B107" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C107" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D107" s="9">
+        <v>338</v>
+      </c>
+      <c r="E107" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A108" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B108" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C108" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D108" s="9">
+        <v>340</v>
+      </c>
+      <c r="E108" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A109" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B109" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C109" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D109" s="9">
+        <v>342</v>
+      </c>
+      <c r="E109" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A110" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B110" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C110" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D110" s="9">
+        <v>344</v>
+      </c>
+      <c r="E110" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A112" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B112" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C112" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D112" s="9">
+        <v>122</v>
+      </c>
+      <c r="E112" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A113" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B113" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C113" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D113" s="9">
+        <v>123</v>
+      </c>
+      <c r="E113" s="9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A114" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B114" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C114" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="D114" s="9">
+        <v>126</v>
+      </c>
+      <c r="E114" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A115" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B115" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C115" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="D115" s="9">
+        <v>138</v>
+      </c>
+      <c r="E115" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A117" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B117" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C117" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D117" s="9">
+        <v>170</v>
+      </c>
+      <c r="E117" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A118" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B118" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C118" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D118" s="9">
+        <v>172</v>
+      </c>
+      <c r="E118" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A119" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B119" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C119" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D119" s="9">
+        <v>174</v>
+      </c>
+      <c r="E119" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A120" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B120" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C120" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D120" s="9">
+        <v>176</v>
+      </c>
+      <c r="E120" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A121" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B121" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C121" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D121" s="9">
+        <v>178</v>
+      </c>
+      <c r="E121" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A122" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B122" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C122" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D122" s="9">
+        <v>180</v>
+      </c>
+      <c r="E122" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A123" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B123" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C123" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D123" s="9">
+        <v>182</v>
+      </c>
+      <c r="E123" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A124" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B124" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C124" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D124" s="9">
+        <v>184</v>
+      </c>
+      <c r="E124" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A125" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B125" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C125" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D125" s="9">
+        <v>186</v>
+      </c>
+      <c r="E125" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A126" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B126" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="C126" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D126" s="9">
+        <v>188</v>
+      </c>
+      <c r="E126" s="9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>